<commit_message>
Revise the Siena valuation for the agent's equipment ages.
The roof is 20 years old, one air conditioner is from 2024, the second is from 2017, and the pool heater is from 2020. Supported value is $880,000, with an $850,000 offer and a $910,000 ceiling.

Co-authored-by: beachbobby45 <beachbobby45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/real_estate/lakewood-ranch-homes.xlsx
+++ b/real_estate/lakewood-ranch-homes.xlsx
@@ -17,13 +17,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subject'!$A$1:$C$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subject'!$A$1:$C$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Subject'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comps'!$A$1:$R$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Comps'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Valuation'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Carrying costs'!$3:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Upgrades'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Upgrades'!$A$1:$D$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Upgrades'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Risks'!$A$1:$D$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Risks'!$1:$1</definedName>
@@ -248,10 +248,10 @@
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1111,68 +1111,85 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Tile, year not stated</t>
+          <t>Tile, 20 years old</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>A 2006 tile roof can still look fine while the underlayment is at the end of its life.</t>
+          <t>Listing agent, 23 Oct 2026. On a 2006 house this is the original roof. Underlayment is the insurance issue. Planning range to replace tile is $40,000–$80,000, not a bid.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Pool</t>
+          <t>HVAC</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Heated in-ground pool and spa, screen cage, outdoor kitchen</t>
+          <t>2024 and 2017</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>All of this was already in the May 2019 listing remarks.</t>
+          <t>Listing agent, 23 Oct 2026. Two systems, replaced on different dates. The 2017 unit is mid-life. Tonnage and zones are still unknown.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Orientation</t>
+          <t>Pool</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Front faces east</t>
+          <t>Heater 2020. Surface and cage undated.</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Photo captions describe a west-facing lanai and sunsets. Consistent with a rear-west plan.</t>
+          <t>The pool, spa, and outdoor kitchen were already in the May 2019 remarks. The heater date does not date the surface or the screen cage.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Orientation</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Front faces east</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Photo captions describe a west-facing lanai and sunsets. Consistent with a rear-west plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
           <t>Schools</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Willis / Nolan / Lakewood Ranch High</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Public assignment. Confirm boundaries before relying on them.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C22"/>
+  <autoFilter ref="A1:C23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -1380,7 +1397,7 @@
       </c>
       <c r="Q2" s="10" t="inlineStr">
         <is>
-          <t>Interior remodel claimed; roof, AC, and water heater not dated</t>
+          <t>Agent 23 Oct 2026: roof 20 years old, HVAC 2024 and HVAC 2017, pool heater 2020. Water heater still undated.</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -2248,7 +2265,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs. The opinion is conditional on the roof and the air conditioner. It is not an appraisal and it is not a prediction of the contract price.</t>
+          <t>Yellow cells are inputs. Updated 23 Oct 2026 for the listing agent's ages: roof 20 years, HVAC 2024 and 2017, pool heater 2020. It is not an appraisal and it is not a prediction of the contract price.</t>
         </is>
       </c>
     </row>
@@ -2394,52 +2411,52 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>Low value, original roof and AC</t>
+          <t>Opening offer</t>
         </is>
       </c>
       <c r="B13" s="32" t="n">
-        <v>860000</v>
+        <v>850000</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Near the size-adjusted 2026 sales, with a reserve for a 2006 roof and AC</t>
+          <t>Start here. The roof is confirmed 20 years old, so the offer leaves room for a roof credit.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Mid value, systems still have life</t>
+          <t>Supported value</t>
         </is>
       </c>
       <c r="B14" s="32" t="n">
-        <v>940000</v>
+        <v>880000</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>About 6% per foot over the 13978 ask, for a newer interior only</t>
+          <t>About the 13978 contract rate on this living area. The 2024 HVAC offsets part of the known roof. It does not support a premium.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>High value, roof and AC are recent</t>
+          <t>Ceiling</t>
         </is>
       </c>
       <c r="B15" s="32" t="n">
-        <v>1030000</v>
+        <v>910000</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Still under the failed $400+/sf tests on this street</t>
+          <t>Only with an affordable insurance binder and a roof report that does not require immediate replacement.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Ask vs mid</t>
+          <t>Ask vs supported</t>
         </is>
       </c>
       <c r="B16" s="33">
@@ -2448,14 +2465,14 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Percent the ask sits above the mid desk value</t>
+          <t>Percent the ask sits above the supported value</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>Dollars above mid</t>
+          <t>Dollars above supported</t>
         </is>
       </c>
       <c r="B17" s="5">
@@ -2464,7 +2481,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Negotiation gap if the mid case holds</t>
+          <t>Gap between the ask and the supported value</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2557,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot.</t>
+          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. On 23 Oct 2026 the listing agent dated the roof at 20 years old, one air conditioner at 2024, the second air conditioner at 2017, and the pool heater at 2020. The 2024 system and the 2020 heater remove the all-original mechanicals case. The 20-year roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000.</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3028,7 +3045,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Already there in 2019. Age of surface, heater, and cage is unknown.</t>
+          <t>Already there in 2019. Heater is 2020 per the agent. Surface and cage are still undated.</t>
         </is>
       </c>
     </row>
@@ -3172,29 +3189,29 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Tile. No year.</t>
+          <t>Agent: 20 years old</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Not described as new in 2019 either</t>
-        </is>
-      </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>Open risk. Underlayment on a 2006 tile roof is the expensive item.</t>
+          <t>Not described as new in 2019</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Original 2006 tile roof. Underlayment is the expensive item. Still get the certification.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Air conditioner</t>
+          <t>Air conditioners</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Central air. No year.</t>
+          <t>Agent: one system 2024, second system 2017</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -3202,80 +3219,102 @@
           <t>Not dated in 2019</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr">
-        <is>
-          <t>Open risk. Neighbors are advertising 2023–2026 replacements.</t>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Two systems. The 2024 unit is current. The 2017 unit is mid-life. Ask which zone each serves.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Water heater</t>
+          <t>Pool heater</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Agent: 2020</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="D17" s="37" t="inlineStr">
-        <is>
-          <t>Open risk. Typical life is inside the time since 2006.</t>
+          <t>Pool and spa already existed</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Serviceable. This date does not cover the pool surface or the screen cage.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Water heater</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Blinds and treatments only</t>
+          <t>Still not dated</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Not described as impact</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>No wind-mitigation credit is being claimed. Verify.</t>
+          <t>Still open. Typical life is inside the time since 2006.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Blinds and treatments only</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Not described as impact</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>No wind-mitigation credit is being claimed. Verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Public record renovation year</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Remarks say fully remodeled, no date</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Redfin shows a 2012 renovation year</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Do not treat 2012 as proven. Pull the permit file.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D19"/>
+  <autoFilter ref="A1:D20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -3332,7 +3371,7 @@
           <t>Price</t>
         </is>
       </c>
-      <c r="B2" s="38" t="inlineStr">
+      <c r="B2" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3344,7 +3383,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Do not write at the ask. Mid desk value is $940,000 only if the roof and AC still have life.</t>
+          <t>Do not write at the ask. Supported value is $880,000. Open at $850,000. Ceiling is $910,000.</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3393,7 @@
           <t>Resale</t>
         </is>
       </c>
-      <c r="B3" s="38" t="inlineStr">
+      <c r="B3" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3376,41 +3415,41 @@
           <t>Roof and insurance</t>
         </is>
       </c>
-      <c r="B4" s="38" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tile roof, house built 2006, year not disclosed. 13828, which sold at $346/sf, led with a brand-new roof.</t>
+          <t>Listing agent says the roof is 20 years old, so it is the original 2006 tile roof. 13828, which sold at $346/sf, led with a brand-new roof.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Roof certification with underlayment age, 4-point, wind mitigation, and an insurance binder before the inspection period ends. Planning range to replace a tile roof of this size is $40,000–$80,000. That is not a bid.</t>
+          <t>Roof certification, 4-point, wind mitigation, and an insurance binder before the inspection period ends. Planning range to replace a tile roof of this size is $40,000–$80,000. That is not a bid.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Air conditioner and water heater</t>
+          <t>Second HVAC and water heater</t>
         </is>
       </c>
       <c r="B5" s="38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Listing is silent. 13853, 13860, 13861, 13911, and 13978 all date a recent HVAC or water heater.</t>
+          <t>Listing agent: one air conditioner replaced in 2024, the second in 2017. Water heater is still undated.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>4-point ages. Planning range for a 4-ton replacement is $8,000–$16,000, water heater $1,500–$3,000. Not bids.</t>
+          <t>Confirm tonnage and which zone each system serves. Budget the 2017 unit for replacement later in the decade. Water heater planning range is $1,500–$3,000 if it is original.</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3459,7 @@
           <t>Tax reset</t>
         </is>
       </c>
-      <c r="B6" s="38" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3442,7 +3481,7 @@
           <t>Remodel story</t>
         </is>
       </c>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3464,7 +3503,7 @@
           <t>HOA disclosure</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3486,14 +3525,14 @@
           <t>Pool and cage</t>
         </is>
       </c>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Marketed as heated pool and spa. No surface, equipment, or cage date. A 2006 aluminum cage in Florida corrodes.</t>
+          <t>Listing agent dated the pool heater at 2020. Surface, pump, and the 2006 screen cage are still undated.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3508,7 +3547,7 @@
           <t>Three bedrooms</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3530,7 +3569,7 @@
           <t>Golf lot</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
Confirm the Siena equipment dates against Manatee permits.
The public file supports the original 2006 tile roof and one 2024 HVAC changeout. The agent's 2017 system and 2020 pool heater are not in the county records, so the brief no longer treats them as credits.

Co-authored-by: beachbobby45 <beachbobby45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/real_estate/lakewood-ranch-homes.xlsx
+++ b/real_estate/lakewood-ranch-homes.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrying costs" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upgrades" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Permits" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subject'!$A$1:$C$23</definedName>
@@ -27,8 +28,10 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Upgrades'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Risks'!$A$1:$D$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Risks'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$1:$C$15</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Sources'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Permits'!$A$4:$G$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Permits'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sources'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Sources'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -774,7 +777,7 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Add the next house as a new row on the Comps sheet. Set Role to Subject, Active, or Sold. Price per living sq ft and the gap versus 13994 calculate themselves. Yellow cells on Valuation are the only inputs. Use living area, never total under-roof area. 13394 Siena Loop is not a parcel; this file analyzes 13994 Siena Loop. Pulled 23 Oct 2026 (Pacific). Desk comparison, not an appraisal.</t>
+          <t>Add the next house as a new row on the Comps sheet. Set Role to Subject, Active, or Sold. Price per living sq ft and the gap versus 13994 calculate themselves. Yellow cells on Valuation are the only inputs. Use living area, never total under-roof area. 13394 Siena Loop is not a parcel; this file analyzes 13994 Siena Loop. The Permits sheet is the Manatee County check of the agent's equipment dates. Pulled 23 Oct 2026 (Pacific). Desk comparison, not an appraisal.</t>
         </is>
       </c>
     </row>
@@ -956,7 +959,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Stucco on slab. Builder not named in the current MLS remarks.</t>
+          <t>Permit CMP-05031188 completed 28 Feb 2006. Neal Communities of Southwest Florida. Concrete block, tile roof, gas.</t>
         </is>
       </c>
     </row>
@@ -990,7 +993,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Manatee County. Zoning A/WPE. Flood zone X on the Coldwell Banker detail page.</t>
+          <t>Listing says zoning A/WPE. The 2024 Accela record says PD-MU. Flood zone X on both.</t>
         </is>
       </c>
     </row>
@@ -1111,12 +1114,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Tile, 20 years old</t>
+          <t>Original tile, completed 28 Feb 2006</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Listing agent, 23 Oct 2026. On a 2006 house this is the original roof. Underlayment is the insurance issue. Planning range to replace tile is $40,000–$80,000, not a bid.</t>
+          <t>CMP-05031188. No reroof permit in the 2006–2018 archive or the live GIS layer. The agent's 20-year age matches. Planning range to replace tile is $40,000–$80,000, not a bid.</t>
         </is>
       </c>
     </row>
@@ -1128,12 +1131,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2024 and 2017</t>
+          <t>One permitted changeout, 30 May 2024</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Listing agent, 23 Oct 2026. Two systems, replaced on different dates. The 2017 unit is mid-life. Tonnage and zones are still unknown.</t>
+          <t>BLD2405-3790, like for like, $9,524, Arctic Air. GIS certificate date 22 May 2026. Accela lists no completed inspections. No permit was found for the agent's 2017 system.</t>
         </is>
       </c>
     </row>
@@ -1145,12 +1148,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Heater 2020. Surface and cage undated.</t>
+          <t>Original pool and cage, 2006</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>The pool, spa, and outdoor kitchen were already in the May 2019 remarks. The heater date does not date the surface or the screen cage.</t>
+          <t>Pool completed 25 May 2006 (CMP-05070213). Mansard cage completed 7 Mar 2006 (CMP-06011072). No 2020 heater permit was found.</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1400,7 @@
       </c>
       <c r="Q2" s="10" t="inlineStr">
         <is>
-          <t>Agent 23 Oct 2026: roof 20 years old, HVAC 2024 and HVAC 2017, pool heater 2020. Water heater still undated.</t>
+          <t>Permits: original tile roof completed 28 Feb 2006 (CMP-05031188). One HVAC changeout issued 30 May 2024 (BLD2405-3790). No 2017 HVAC permit and no 2020 pool-heater permit.</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -2262,10 +2265,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs. Updated 23 Oct 2026 for the listing agent's ages: roof 20 years, HVAC 2024 and 2017, pool heater 2020. It is not an appraisal and it is not a prediction of the contract price.</t>
+          <t>Yellow cells are inputs. Updated 23 Oct 2026 after a Manatee County permit check. The roof is the original tile roof, completed 28 Feb 2006. One HVAC changeout was permitted on 30 May 2024. The agent's 2017 HVAC date and 2020 pool-heater date are not in the public permit file. It is not an appraisal and it is not a prediction of the contract price.</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2422,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Start here. The roof is confirmed 20 years old, so the offer leaves room for a roof credit.</t>
+          <t>Start here. The roof permit confirms original tile completed 28 Feb 2006, so the offer leaves room for a roof credit.</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2437,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>About the 13978 contract rate on this living area. The 2024 HVAC offsets part of the known roof. It does not support a premium.</t>
+          <t>About the 13978 contract rate on this living area. One permitted 2024 changeout offsets part of the roof. It does not support a premium, and the unconfirmed 2017 system does not add value.</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2452,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Only with an affordable insurance binder and a roof report that does not require immediate replacement.</t>
+          <t>Only with an affordable insurance binder, a roof report that does not require immediate replacement, and a data plate or invoice showing the second system is 2017 or newer.</t>
         </is>
       </c>
     </row>
@@ -2554,16 +2557,16 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. On 23 Oct 2026 the listing agent dated the roof at 20 years old, one air conditioner at 2024, the second air conditioner at 2017, and the pool heater at 2020. The 2024 system and the 2020 heater remove the all-original mechanicals case. The 20-year roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1"/>
-    <row r="26" ht="30" customHeight="1"/>
-    <row r="27" ht="30" customHeight="1"/>
+          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000 unless the second system's data plate is 2017 or newer and the roof report is clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1"/>
+    <row r="26" ht="36" customHeight="1"/>
+    <row r="27" ht="36" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A24:C27"/>
@@ -3045,7 +3048,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Already there in 2019. Heater is 2020 per the agent. Surface and cage are still undated.</t>
+          <t>Original. Pool completed 25 May 2006. Cage completed 7 Mar 2006. No later permit.</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3202,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Original 2006 tile roof. Underlayment is the expensive item. Still get the certification.</t>
+          <t>Confirmed original. CMP-05031188 completed 28 Feb 2006. No reroof permit. Still get the certification.</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3224,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Two systems. The 2024 unit is current. The 2017 unit is mid-life. Ask which zone each serves.</t>
+          <t>One permit only: BLD2405-3790, issued 30 May 2024, like for like, $9,524. No 2017 permit. Require the second data plate.</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3246,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Serviceable. This date does not cover the pool surface or the screen cage.</t>
+          <t>No heater permit in the live county layer. Do not pay for a 2020 heater without the invoice or data plate.</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3268,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Still open. Typical life is inside the time since 2006.</t>
+          <t>No water-heater permit in the files searched. Planning range is $1,500–$3,000 if it is original.</t>
         </is>
       </c>
     </row>
@@ -3309,7 +3312,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Do not treat 2012 as proven. Pull the permit file.</t>
+          <t>No kitchen, bath, or alteration permit was found for this parcel. Do not treat 2012 as proven.</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3425,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Listing agent says the roof is 20 years old, so it is the original 2006 tile roof. 13828, which sold at $346/sf, led with a brand-new roof.</t>
+          <t>Permit CMP-05031188 completed 28 Feb 2006 with a tile roof. No reroof permit follows it. 13828, which sold at $346/sf, led with a brand-new roof.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -3437,19 +3440,19 @@
           <t>Second HVAC and water heater</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="B5" s="37" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Listing agent: one air conditioner replaced in 2024, the second in 2017. Water heater is still undated.</t>
+          <t>The only HVAC permit is BLD2405-3790, one like-for-like changeout issued 30 May 2024 for $9,524. No 2017 permit was found. No water-heater permit was found.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Confirm tonnage and which zone each system serves. Budget the 2017 unit for replacement later in the decade. Water heater planning range is $1,500–$3,000 if it is original.</t>
+          <t>Read both data plates. If the second system is original, budget a replacement. Water heater planning range is $1,500–$3,000 if it is original. Accela lists no completed inspections on the 2024 permit; GIS shows a certificate date of 22 May 2026.</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3491,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2019 remarks already included the pool, spa, outdoor kitchen, tile, tall cabinets, granite, and office bath. Redfin shows a 2012 renovation field.</t>
+          <t>2019 remarks already included the pool, spa, outdoor kitchen, tile, tall cabinets, granite, and office bath. The county files checked have no kitchen, bath, or alteration permit. Redfin's 2012 field is not a permit.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Permit search for kitchen, bath, electric, and any wall changes. Unpermitted work is a loan and insurance problem.</t>
+          <t>Do not pay a remodel premium the permit file does not support. Ask the seller for invoices. Unpermitted work is a loan and insurance problem.</t>
         </is>
       </c>
     </row>
@@ -3532,12 +3535,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Listing agent dated the pool heater at 2020. Surface, pump, and the 2006 screen cage are still undated.</t>
+          <t>Pool completed 25 May 2006. Mansard cage completed 7 Mar 2006. No later pool, heater, or cage permit. The agent's 2020 heater date is not in the county file.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Pool inspection. Resurface and rescreen are separate five-figure and four-figure jobs when they are due.</t>
+          <t>Pool inspection. Do not credit a 2020 heater without the data plate or invoice. Resurface and rescreen are separate jobs when they are due.</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3702,329 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Manatee County public permits for 13994 Siena Loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Checked 23 Oct 2026. Archive CSVs published by Manatee Development Services cover 2004 through 21 Feb 2018. The live GIS PermitData layer, queried by parcel 588502359 and by house 13994 SIENA, returned one building permit, BLD2405-3790, plus a pointer to the historical archive. A missing permit means it was not in those public files. It does not prove the equipment was never replaced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Permit</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Issued</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>What the county file shows</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Against the agent's date</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>New house and tile roof</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>CMP-05031188</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>28 Mar 2005</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>28 Feb 2006</t>
+        </is>
+      </c>
+      <c r="E5" s="39" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Original 3-bed, 3-bath, one-story concrete-block house with a tile roof and gas. Neal Communities of Southwest Florida. Declared cost $130,000. Lot 47.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Matches the agent's 20-year roof. No reroof permit appears after this one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pool and spa</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>CMP-05070213</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>4 Aug 2005</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>25 May 2006</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In-ground pool, spa, and deck. Splash Pools. Declared cost $28,100. Built with the house.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>The pool is original. This permit does not date a heater.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Screen cage</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>CMP-06011072</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>23 Feb 2006</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>7 Mar 2006</t>
+        </is>
+      </c>
+      <c r="E7" s="39" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Mansard pool cage on the existing deck. Absolute Aluminum. Declared cost $6,667.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>The cage is original. No later cage or rescreen permit was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Air conditioner</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>BLD2405-3790</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>30 May 2024</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>GIS certificate 22 May 2026</t>
+        </is>
+      </c>
+      <c r="E8" s="39" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>One like-for-like HVAC changeout. Arctic Air Services, Scott Whitaker. Job value $9,524. No duct replacement. Mechanical only. Accela lists no completed inspections.</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Confirms one 2024 system, not two. The agent's 2017 system has no permit in the files searched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Second air conditioner, 2017</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Not in file</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>No 2017 mechanical permit for this parcel in the 2013–2018 archive or in the live GIS layer.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>The 2017 date is the agent's statement only. The second system may still be the 2006 equipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Pool heater, 2020</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>Not in file</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>A 2020 heater permit would be in the live Accela-era layer. That layer has no heater permit for this house.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>The 2020 heater date is the agent's statement only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Kitchen, baths, water heater</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Not in file</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>No alteration, plumbing, or water-heater permit for this parcel in the files searched. Redfin's 2012 renovation year is not a permit.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Finish claims are not backed by a county building permit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G11"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LCounty permits, parcel 588502359</oddHeader>
+    <oddFooter>&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -3958,12 +4283,97 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Unverified county field</t>
+          <t>Not matched to a permit</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>New house and tile roof, completed 28 Feb 2006</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Manatee historical permit CMP-05031188, parcel 588502359</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Archive file 2004–2005, checked 23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Pool and spa, completed 25 May 2006</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Manatee historical permit CMP-05070213</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Archive file 2004–2005, checked 23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Mansard screen cage, completed 7 Mar 2006</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Manatee historical permit CMP-06011072</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Archive file 2006, checked 23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>One HVAC changeout, issued 30 May 2024, GIS certificate 22 May 2026</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Manatee GIS PermitData and Accela BLD2405-3790</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Live layer and Accela page, 23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>No 2017 HVAC permit, no 2020 heater permit, no remodel permit</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Same archive CSVs through 21 Feb 2018, plus the live GIS layer for this parcel and house</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Checked 23 Oct 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:C20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Record two rejected offers under $1 million.
The listing agent told our broker the owners turned down both. The desk range stays at $850,000, $880,000, and $910,000, because those rejections do not support paying $1,000,000.

Co-authored-by: beachbobby45 <beachbobby45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/real_estate/lakewood-ranch-homes.xlsx
+++ b/real_estate/lakewood-ranch-homes.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Risks'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Permits'!$A$4:$G$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Permits'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sources'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sources'!$A$1:$C$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Sources'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -860,12 +860,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Active, 49 days, no cut</t>
+          <t>Active, 49 days, two offers rejected</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Zachos snapshot updated 23 Oct 2026. An open house was scheduled 18 Oct 2026, 1–4pm.</t>
+          <t>No price cut. The listing agent told our broker the owners rejected two offers, both under $1,000,000. The amounts were not disclosed.</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Start here. The roof permit confirms original tile completed 28 Feb 2006, so the offer leaves room for a roof credit.</t>
+          <t>Start here. The owners have already rejected two offers under $1,000,000, so this number may be refused. The roof permit still calls for the credit. Do not raise it to meet a counter at $1,000,000.</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000 unless the second system's data plate is 2017 or newer and the roof report is clean.</t>
+          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000 unless the second system's data plate is 2017 or newer and the roof report is clean. On 23 Oct 2026 the listing agent told our broker the owners have rejected two offers, both under $1,000,000. The amounts were not disclosed. That confirms buyers are writing below $1,000,000. It is not a reason to pay $1,000,000. A counter at or above $1,000,000 is still above the comps.</t>
         </is>
       </c>
     </row>
@@ -3381,12 +3381,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Ask is $456/sf against a 2026 sold median near $314/sf and a same-view neighbor under contract at $336/sf.</t>
+          <t>Ask is $456/sf against a 2026 sold median near $314/sf and a same-view neighbor under contract at $336/sf. The owners rejected two offers under $1,000,000. Amounts were not disclosed.</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Do not write at the ask. Supported value is $880,000. Open at $850,000. Ceiling is $910,000.</t>
+          <t>Do not write at the ask, and do not raise the bid because those offers were rejected. Supported value is $880,000. Open at $850,000. Ceiling is $910,000. A counter at or above $1,000,000 is still above the comps.</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -4372,8 +4372,25 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Two offers under $1,000,000, both rejected</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Listing agent, told to our broker. Dollar amounts were not disclosed</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Recommend passing on 13994 Siena Loop.
The owners rejected two offers under $1 million and are still asking $1,195,000. A bid at the comp range would ask them to take a price they have already refused.

Co-authored-by: beachbobby45 <beachbobby45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/real_estate/lakewood-ranch-homes.xlsx
+++ b/real_estate/lakewood-ranch-homes.xlsx
@@ -2265,10 +2265,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs. Updated 23 Oct 2026 after a Manatee County permit check. The roof is the original tile roof, completed 28 Feb 2006. One HVAC changeout was permitted on 30 May 2024. The agent's 2017 HVAC date and 2020 pool-heater date are not in the public permit file. It is not an appraisal and it is not a prediction of the contract price.</t>
+          <t>Yellow cells are inputs. Recommendation on 23 Oct 2026 is to pass. The owners rejected two offers under $1,000,000 and are still asking $1,195,000. The roof is the original tile roof, completed 28 Feb 2006. One HVAC changeout was permitted on 30 May 2024. The agent's 2017 HVAC date and 2020 pool-heater date are not in the public permit file. It is not an appraisal and it is not a prediction of the contract price.</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>Opening offer</t>
+          <t>Pass unless the price is</t>
         </is>
       </c>
       <c r="B13" s="32" t="n">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Start here. The owners have already rejected two offers under $1,000,000, so this number may be refused. The roof permit still calls for the credit. Do not raise it to meet a counter at $1,000,000.</t>
+          <t>No offer today. The owners rejected two bids under $1,000,000 and are still asking $1,195,000. This cell is the bottom of the old bid range, not an instruction to write it.</t>
         </is>
       </c>
     </row>
@@ -2444,7 +2444,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>Ceiling</t>
+          <t>Reopen the file at or below</t>
         </is>
       </c>
       <c r="B15" s="32" t="n">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Only with an affordable insurance binder, a roof report that does not require immediate replacement, and a data plate or invoice showing the second system is 2017 or newer.</t>
+          <t>Only if the ask or a written counter is this or less, with an affordable insurance binder, a roof report that does not require immediate replacement, and a data plate showing the second system is 2017 or newer.</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. Open at $850,000. Do not exceed $910,000 unless the second system's data plate is 2017 or newer and the roof report is clean. On 23 Oct 2026 the listing agent told our broker the owners have rejected two offers, both under $1,000,000. The amounts were not disclosed. That confirms buyers are writing below $1,000,000. It is not a reason to pay $1,000,000. A counter at or above $1,000,000 is still above the comps.</t>
+          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. On 23 Oct 2026 the listing agent told our broker the owners have rejected two offers, both under $1,000,000. The amounts were not disclosed. The owners are holding a price above the bids buyers will write. Pass. Reopen the file only if the ask or a written counter is $910,000 or less.</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Do not write at the ask, and do not raise the bid because those offers were rejected. Supported value is $880,000. Open at $850,000. Ceiling is $910,000. A counter at or above $1,000,000 is still above the comps.</t>
+          <t>Pass. The owners rejected the band buyers are writing. Supported value is $880,000. Reopen the file only if the ask or a counter is $910,000 or less.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wait for a list price under $1 million before offering.
No offer has been sent, so there is no counter to watch. The bid to write after that list cut is still $850,000 to $910,000.

Co-authored-by: beachbobby45 <beachbobby45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/real_estate/lakewood-ranch-homes.xlsx
+++ b/real_estate/lakewood-ranch-homes.xlsx
@@ -2268,7 +2268,7 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs. Recommendation on 23 Oct 2026 is to pass. The owners rejected two offers under $1,000,000 and are still asking $1,195,000. The roof is the original tile roof, completed 28 Feb 2006. One HVAC changeout was permitted on 30 May 2024. The agent's 2017 HVAC date and 2020 pool-heater date are not in the public permit file. It is not an appraisal and it is not a prediction of the contract price.</t>
+          <t>Yellow cells are inputs. No offer has been sent. Wait until the list price is under $1,000,000, then write $850,000 to $910,000. The owners rejected two other offers under $1,000,000 and are still asking $1,195,000. The roof is the original tile roof, completed 28 Feb 2006. One HVAC changeout was permitted on 30 May 2024. The agent's 2017 HVAC date and 2020 pool-heater date are not in the public permit file. It is not an appraisal and it is not a prediction of the contract price.</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>Pass unless the price is</t>
+          <t>Opening offer, once listed under $1,000,000</t>
         </is>
       </c>
       <c r="B13" s="32" t="n">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>No offer today. The owners rejected two bids under $1,000,000 and are still asking $1,195,000. This cell is the bottom of the old bid range, not an instruction to write it.</t>
+          <t>No offer has been sent. This number is what to write after the list price falls under $1,000,000. It is not an offer to send at the current ask.</t>
         </is>
       </c>
     </row>
@@ -2444,7 +2444,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>Reopen the file at or below</t>
+          <t>Ceiling once listed under $1,000,000</t>
         </is>
       </c>
       <c r="B15" s="32" t="n">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Only if the ask or a written counter is this or less, with an affordable insurance binder, a roof report that does not require immediate replacement, and a data plate showing the second system is 2017 or newer.</t>
+          <t>Top of the offer after the list price is under $1,000,000. Still requires an affordable insurance binder, a roof report that does not require immediate replacement, and a data plate showing the second system is 2017 or newer.</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. On 23 Oct 2026 the listing agent told our broker the owners have rejected two offers, both under $1,000,000. The amounts were not disclosed. The owners are holding a price above the bids buyers will write. Pass. Reopen the file only if the ask or a written counter is $910,000 or less.</t>
+          <t>Six 2026 sales on this loop closed from $286 to $346 per living foot, median about $314. The four active neighbors are $298 to $336 per foot. The closest product, 13978, has the same bedroom count, three baths, an office, and a golf-and-lake lot, plus a dated April 2026 air conditioner, and it found a buyer at a $899,000 ask. Sizing that rate to 2,623 feet is about $882,000. 13911 started at $1,295,000 in January 2026, has been cut to $995,000, and was still active in August with more bedrooms, more baths, and a 2024 air conditioner. This house's own 2019 campaign listed at $540,000 and sold at $445,000. The current remarks sell a remodel. The May 2019 remarks already advertised the pool, spa, outdoor kitchen, tile floors, 48-inch cabinets, granite island, and the office bath. Quartz, new cabinet claims, bath glass, a wine bar, an electric fireplace, and a softener can support a finish premium. They do not support $456 per foot. Manatee permits confirm the tile roof is original: CMP-05031188 was completed 28 Feb 2006, and no reroof permit follows it. The only later mechanical permit is BLD2405-3790, a like-for-like HVAC changeout issued 30 May 2024 for $9,524. That is one system. The agent's 2017 air conditioner and 2020 pool heater are not in the county file, so they are not credits. The original roof removes the $1,030,000 case. Supported value is $880,000. On 23 Oct 2026 the listing agent told our broker the owners have rejected two offers, both under $1,000,000. The amounts were not disclosed. The owners are holding a price above the bids buyers will write. No offer has been sent. Wait until the house is listed under $1,000,000, then write $850,000 to $910,000.</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Pass. The owners rejected the band buyers are writing. Supported value is $880,000. Reopen the file only if the ask or a counter is $910,000 or less.</t>
+          <t>No offer has been sent. Wait until the list price is under $1,000,000, then write $850,000 to $910,000. Supported value is $880,000.</t>
         </is>
       </c>
     </row>

</xml_diff>